<commit_message>
update: descripción del cambio
</commit_message>
<xml_diff>
--- a/data/database.xlsx
+++ b/data/database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nelso\futbol-app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BEEF761-8E07-4634-BB50-4CE5A9848989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A911B01-9038-41AA-82B1-3BFCD504458D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1762,9 +1762,6 @@
     <t>M. Klimowicz</t>
   </si>
   <si>
-    <t>AMF, LCMF, RW</t>
-  </si>
-  <si>
     <t>Argentina, Germany</t>
   </si>
   <si>
@@ -1916,6 +1913,9 @@
   </si>
   <si>
     <t>P. Álvarez</t>
+  </si>
+  <si>
+    <t>LCMF, RW</t>
   </si>
 </sst>
 </file>
@@ -96640,7 +96640,7 @@
         <v>118</v>
       </c>
       <c r="D307" t="s">
-        <v>580</v>
+        <v>631</v>
       </c>
       <c r="E307">
         <v>25</v>
@@ -96679,7 +96679,7 @@
         <v>120</v>
       </c>
       <c r="Q307" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="R307" t="s">
         <v>107</v>
@@ -96939,7 +96939,7 @@
     </row>
     <row r="308" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B308" t="s">
         <v>111</v>
@@ -97247,7 +97247,7 @@
     </row>
     <row r="309" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B309" t="s">
         <v>111</v>
@@ -97555,7 +97555,7 @@
     </row>
     <row r="310" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B310" t="s">
         <v>111</v>
@@ -97564,7 +97564,7 @@
         <v>111</v>
       </c>
       <c r="D310" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="E310">
         <v>20</v>
@@ -97863,7 +97863,7 @@
     </row>
     <row r="311" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B311" t="s">
         <v>111</v>
@@ -98171,7 +98171,7 @@
     </row>
     <row r="312" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B312" t="s">
         <v>111</v>
@@ -98479,7 +98479,7 @@
     </row>
     <row r="313" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B313" t="s">
         <v>111</v>
@@ -98488,7 +98488,7 @@
         <v>111</v>
       </c>
       <c r="D313" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="E313">
         <v>32</v>
@@ -98787,7 +98787,7 @@
     </row>
     <row r="314" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B314" t="s">
         <v>111</v>
@@ -99095,7 +99095,7 @@
     </row>
     <row r="315" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B315" t="s">
         <v>111</v>
@@ -99403,7 +99403,7 @@
     </row>
     <row r="316" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B316" t="s">
         <v>118</v>
@@ -99711,7 +99711,7 @@
     </row>
     <row r="317" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B317" t="s">
         <v>118</v>
@@ -99720,7 +99720,7 @@
         <v>118</v>
       </c>
       <c r="D317" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="E317">
         <v>0</v>
@@ -100019,7 +100019,7 @@
     </row>
     <row r="318" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B318" t="s">
         <v>111</v>
@@ -100327,7 +100327,7 @@
     </row>
     <row r="319" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B319" t="s">
         <v>118</v>
@@ -100336,7 +100336,7 @@
         <v>118</v>
       </c>
       <c r="D319" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="E319">
         <v>18</v>
@@ -100635,7 +100635,7 @@
     </row>
     <row r="320" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B320" t="s">
         <v>111</v>
@@ -100653,7 +100653,7 @@
         <v>0</v>
       </c>
       <c r="G320" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="H320">
         <v>2</v>
@@ -100943,7 +100943,7 @@
     </row>
     <row r="321" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B321" t="s">
         <v>111</v>
@@ -101251,7 +101251,7 @@
     </row>
     <row r="322" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B322" t="s">
         <v>118</v>
@@ -101559,7 +101559,7 @@
     </row>
     <row r="323" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B323" t="s">
         <v>111</v>
@@ -101867,7 +101867,7 @@
     </row>
     <row r="324" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B324" t="s">
         <v>111</v>
@@ -102175,7 +102175,7 @@
     </row>
     <row r="325" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B325" t="s">
         <v>165</v>
@@ -102483,7 +102483,7 @@
     </row>
     <row r="326" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B326" t="s">
         <v>139</v>
@@ -102791,7 +102791,7 @@
     </row>
     <row r="327" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B327" t="s">
         <v>139</v>
@@ -103099,7 +103099,7 @@
     </row>
     <row r="328" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B328" t="s">
         <v>165</v>
@@ -103407,7 +103407,7 @@
     </row>
     <row r="329" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B329" t="s">
         <v>165</v>
@@ -103715,7 +103715,7 @@
     </row>
     <row r="330" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B330" t="s">
         <v>139</v>
@@ -103724,7 +103724,7 @@
         <v>139</v>
       </c>
       <c r="D330" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="E330">
         <v>30</v>
@@ -104023,7 +104023,7 @@
     </row>
     <row r="331" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B331" t="s">
         <v>139</v>
@@ -104331,7 +104331,7 @@
     </row>
     <row r="332" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B332" t="s">
         <v>139</v>
@@ -104340,7 +104340,7 @@
         <v>139</v>
       </c>
       <c r="D332" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="E332">
         <v>19</v>
@@ -104639,7 +104639,7 @@
     </row>
     <row r="333" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B333" t="s">
         <v>165</v>
@@ -104648,7 +104648,7 @@
         <v>165</v>
       </c>
       <c r="D333" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="E333">
         <v>23</v>
@@ -104947,7 +104947,7 @@
     </row>
     <row r="334" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B334" t="s">
         <v>139</v>
@@ -104956,7 +104956,7 @@
         <v>139</v>
       </c>
       <c r="D334" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="E334">
         <v>22</v>
@@ -105255,7 +105255,7 @@
     </row>
     <row r="335" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B335" t="s">
         <v>165</v>
@@ -105563,7 +105563,7 @@
     </row>
     <row r="336" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B336" t="s">
         <v>139</v>
@@ -105871,7 +105871,7 @@
     </row>
     <row r="337" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B337" t="s">
         <v>139</v>
@@ -106179,7 +106179,7 @@
     </row>
     <row r="338" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B338" t="s">
         <v>165</v>
@@ -106487,7 +106487,7 @@
     </row>
     <row r="339" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B339" t="s">
         <v>165</v>
@@ -107103,7 +107103,7 @@
     </row>
     <row r="341" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B341" t="s">
         <v>165</v>
@@ -107411,7 +107411,7 @@
     </row>
     <row r="342" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B342" t="s">
         <v>139</v>
@@ -107719,7 +107719,7 @@
     </row>
     <row r="343" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B343" t="s">
         <v>139</v>
@@ -108027,7 +108027,7 @@
     </row>
     <row r="344" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B344" t="s">
         <v>139</v>
@@ -108335,7 +108335,7 @@
     </row>
     <row r="345" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B345" t="s">
         <v>165</v>
@@ -108344,7 +108344,7 @@
         <v>165</v>
       </c>
       <c r="D345" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="E345">
         <v>27</v>
@@ -108643,7 +108643,7 @@
     </row>
     <row r="346" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B346" t="s">
         <v>165</v>
@@ -108652,7 +108652,7 @@
         <v>165</v>
       </c>
       <c r="D346" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="E346">
         <v>30</v>
@@ -108951,7 +108951,7 @@
     </row>
     <row r="347" spans="1:102" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B347" t="s">
         <v>139</v>

</xml_diff>